<commit_message>
graph updates and add path findings
</commit_message>
<xml_diff>
--- a/AI-Supply-Chain-Network.xlsx
+++ b/AI-Supply-Chain-Network.xlsx
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J98"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
@@ -5312,6 +5312,156 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>SAMBANOVA</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>SambaNova Systems</t>
+        </is>
+      </c>
+      <c r="C96" s="8" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>(private)</t>
+        </is>
+      </c>
+      <c r="E96" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F96" s="8" t="inlineStr">
+        <is>
+          <t>Chip Designers (Accelerators/Networking)</t>
+        </is>
+      </c>
+      <c r="G96" s="8" t="inlineStr">
+        <is>
+          <t>AI accelerators / RDU</t>
+        </is>
+      </c>
+      <c r="H96" s="8" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I96" s="8" t="inlineStr">
+        <is>
+          <t>Reconfigurable Dataflow Units, inference systems</t>
+        </is>
+      </c>
+      <c r="J96" s="8" t="inlineStr">
+        <is>
+          <t>AI-chip designer pairing rack-scale inference systems with Intel Xeon hosts</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>BYTEDANCE</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>ByteDance</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>(private)</t>
+        </is>
+      </c>
+      <c r="E97" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F97" s="8" t="inlineStr">
+        <is>
+          <t>Hyperscalers / Cloud</t>
+        </is>
+      </c>
+      <c r="G97" s="8" t="inlineStr">
+        <is>
+          <t>Hyperscaler (China)</t>
+        </is>
+      </c>
+      <c r="H97" s="8" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="I97" s="8" t="inlineStr">
+        <is>
+          <t>TikTok/Doubao, AI datacenters</t>
+        </is>
+      </c>
+      <c r="J97" s="8" t="inlineStr">
+        <is>
+          <t>China hyperscaler adopting Arm AGI CPU for AI datacenter deployments</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="B98" s="8" t="inlineStr">
+        <is>
+          <t>SpaceX (Colossus compute)</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="E98" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F98" s="8" t="inlineStr">
+        <is>
+          <t>Hyperscalers / Cloud</t>
+        </is>
+      </c>
+      <c r="G98" s="8" t="inlineStr">
+        <is>
+          <t>Neocloud / compute capacity</t>
+        </is>
+      </c>
+      <c r="H98" s="8" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I98" s="8" t="inlineStr">
+        <is>
+          <t>Colossus AI datacenters (Memphis); GPU compute rental</t>
+        </is>
+      </c>
+      <c r="J98" s="8" t="inlineStr">
+        <is>
+          <t>Musk-linked neocloud renting NVDA-GPU compute to Google &amp; Anthropic; IPO ~Jun-2026 (?) Colossus commonly associated with xAI</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J48"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -5326,7 +5476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I226"/>
+  <dimension ref="A1:I238"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
@@ -6602,15 +6752,19 @@
       </c>
       <c r="G30" s="15" t="inlineStr">
         <is>
-          <t>Lead HBM supplier</t>
+          <t>(FACT, X-scan 2026-06-05): Jensen certified SK Hynix for Vera Rubin HBM4 supply (est 60-70% of volume); press-corroborated; lead HBM supplier</t>
         </is>
       </c>
       <c r="H30" s="15" t="inlineStr">
         <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="I30" s="15" t="n"/>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I30" s="15" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-1204-x-scan.md</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="9">
       <c r="A31" s="15" t="inlineStr">
@@ -6909,15 +7063,19 @@
       </c>
       <c r="G37" s="15" t="inlineStr">
         <is>
-          <t>TPU partner</t>
+          <t>(FACT, X-scan 2026-06-05): AVGO Q2 FY26 call - Google TPU commitment 'remains substantial' despite supplier diversification</t>
         </is>
       </c>
       <c r="H37" s="15" t="inlineStr">
         <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="I37" s="15" t="n"/>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I37" s="15" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-1204-x-scan.md</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="9">
       <c r="A38" s="15" t="inlineStr">
@@ -14819,6 +14977,546 @@
       <c r="I226" s="8" t="inlineStr">
         <is>
           <t>ASML.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="8" t="inlineStr">
+        <is>
+          <t>FOXCONN</t>
+        </is>
+      </c>
+      <c r="B227" s="8" t="inlineStr">
+        <is>
+          <t>Foxconn (Hon Hai)</t>
+        </is>
+      </c>
+      <c r="C227" s="8" t="inlineStr">
+        <is>
+          <t>partners with</t>
+        </is>
+      </c>
+      <c r="D227" s="8" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="E227" s="8" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="F227" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G227" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-04): Hon Hai (Foxconn) and Intel announced strategic collaboration on next-gen AI infrastructure, Edge AI, and Physical AI</t>
+        </is>
+      </c>
+      <c r="H227" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="I227" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-04-0404-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="8" t="inlineStr">
+        <is>
+          <t>SAMBANOVA</t>
+        </is>
+      </c>
+      <c r="B228" s="8" t="inlineStr">
+        <is>
+          <t>SambaNova Systems</t>
+        </is>
+      </c>
+      <c r="C228" s="8" t="inlineStr">
+        <is>
+          <t>partners with</t>
+        </is>
+      </c>
+      <c r="D228" s="8" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="E228" s="8" t="inlineStr">
+        <is>
+          <t>Intel</t>
+        </is>
+      </c>
+      <c r="F228" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G228" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-04): SambaNova AI platform paired with Intel Xeon processors in rack-scale infrastructure for hyperscale deployments, disclosed alongside the Foxconn–Intel Computex 2026 announcement.</t>
+        </is>
+      </c>
+      <c r="H228" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="I228" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-04-1204-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="8" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="B229" s="8" t="inlineStr">
+        <is>
+          <t>TSMC</t>
+        </is>
+      </c>
+      <c r="C229" s="8" t="inlineStr">
+        <is>
+          <t>benefits from</t>
+        </is>
+      </c>
+      <c r="D229" s="8" t="inlineStr">
+        <is>
+          <t>T_INFER</t>
+        </is>
+      </c>
+      <c r="E229" s="8" t="inlineStr">
+        <is>
+          <t>AI Inference Demand</t>
+        </is>
+      </c>
+      <c r="F229" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G229" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): C.C. Wei at 6/4 AGM guided 2026 revenue growth &gt;30% USD and 2026 capex near upper end of $52-56B, citing agentic-AI compute/token demand.</t>
+        </is>
+      </c>
+      <c r="H229" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="I229" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-0404-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="8" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B230" s="8" t="inlineStr">
+        <is>
+          <t>Micron</t>
+        </is>
+      </c>
+      <c r="C230" s="8" t="inlineStr">
+        <is>
+          <t>supplies HBM to</t>
+        </is>
+      </c>
+      <c r="D230" s="8" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E230" s="8" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="F230" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G230" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): Jensen certified Micron for Vera Rubin HBM4 supply; press-corroborated</t>
+        </is>
+      </c>
+      <c r="H230" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I230" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-1204-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="8" t="inlineStr">
+        <is>
+          <t>SAMSUNG</t>
+        </is>
+      </c>
+      <c r="B231" s="8" t="inlineStr">
+        <is>
+          <t>Samsung Electronics</t>
+        </is>
+      </c>
+      <c r="C231" s="8" t="inlineStr">
+        <is>
+          <t>supplies HBM to</t>
+        </is>
+      </c>
+      <c r="D231" s="8" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="E231" s="8" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="F231" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G231" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): Jensen certified Samsung for Vera Rubin HBM4 supply; press-corroborated</t>
+        </is>
+      </c>
+      <c r="H231" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I231" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-1204-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="8" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B232" s="8" t="inlineStr">
+        <is>
+          <t>Arm Holdings</t>
+        </is>
+      </c>
+      <c r="C232" s="8" t="inlineStr">
+        <is>
+          <t>licenses CPU IP to</t>
+        </is>
+      </c>
+      <c r="D232" s="8" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="E232" s="8" t="inlineStr">
+        <is>
+          <t>Meta Platforms</t>
+        </is>
+      </c>
+      <c r="F232" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G232" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): Meta named Arm AGI-CPU customer; Arm CEO at Computex, press-corroborated</t>
+        </is>
+      </c>
+      <c r="H232" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I232" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-1204-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="8" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B233" s="8" t="inlineStr">
+        <is>
+          <t>Arm Holdings</t>
+        </is>
+      </c>
+      <c r="C233" s="8" t="inlineStr">
+        <is>
+          <t>licenses CPU IP to</t>
+        </is>
+      </c>
+      <c r="D233" s="8" t="inlineStr">
+        <is>
+          <t>OPENAI</t>
+        </is>
+      </c>
+      <c r="E233" s="8" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="F233" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G233" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): OpenAI in Arm AGI-CPU customer roster; press-corroborated</t>
+        </is>
+      </c>
+      <c r="H233" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I233" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-1204-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="8" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B234" s="8" t="inlineStr">
+        <is>
+          <t>Arm Holdings</t>
+        </is>
+      </c>
+      <c r="C234" s="8" t="inlineStr">
+        <is>
+          <t>licenses CPU IP to</t>
+        </is>
+      </c>
+      <c r="D234" s="8" t="inlineStr">
+        <is>
+          <t>ORCL</t>
+        </is>
+      </c>
+      <c r="E234" s="8" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="F234" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G234" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): Oracle named Arm AGI-CPU adopter at Computex; press-corroborated</t>
+        </is>
+      </c>
+      <c r="H234" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I234" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-1204-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="8" t="inlineStr">
+        <is>
+          <t>ARM</t>
+        </is>
+      </c>
+      <c r="B235" s="8" t="inlineStr">
+        <is>
+          <t>Arm Holdings</t>
+        </is>
+      </c>
+      <c r="C235" s="8" t="inlineStr">
+        <is>
+          <t>licenses CPU IP to</t>
+        </is>
+      </c>
+      <c r="D235" s="8" t="inlineStr">
+        <is>
+          <t>BYTEDANCE</t>
+        </is>
+      </c>
+      <c r="E235" s="8" t="inlineStr">
+        <is>
+          <t>ByteDance</t>
+        </is>
+      </c>
+      <c r="F235" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G235" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): ByteDance named Arm AGI-CPU adopter at Computex; press-corroborated</t>
+        </is>
+      </c>
+      <c r="H235" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I235" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-1204-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="8" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="B236" s="8" t="inlineStr">
+        <is>
+          <t>Alphabet (Google)</t>
+        </is>
+      </c>
+      <c r="C236" s="8" t="inlineStr">
+        <is>
+          <t>runs compute on</t>
+        </is>
+      </c>
+      <c r="D236" s="8" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="E236" s="8" t="inlineStr">
+        <is>
+          <t>SpaceX (Colossus compute)</t>
+        </is>
+      </c>
+      <c r="F236" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G236" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): Google to rent ~$30B / ~110k NVDA-GPU compute capacity from SpaceX (Colossus), $920M/mo Oct-2026-&gt;Jun-2029; multi-press (?) Colossus usually attributed to xAI</t>
+        </is>
+      </c>
+      <c r="H236" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I236" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-2004-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="8" t="inlineStr">
+        <is>
+          <t>ANTHROPIC</t>
+        </is>
+      </c>
+      <c r="B237" s="8" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C237" s="8" t="inlineStr">
+        <is>
+          <t>runs compute on</t>
+        </is>
+      </c>
+      <c r="D237" s="8" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="E237" s="8" t="inlineStr">
+        <is>
+          <t>SpaceX (Colossus compute)</t>
+        </is>
+      </c>
+      <c r="F237" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G237" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): Anthropic ~$45B multiyear compute deal across SpaceX Colossus / Colossus II ($1.25B/mo through May-2029) (?) Colossus usually attributed to xAI</t>
+        </is>
+      </c>
+      <c r="H237" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I237" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-2004-x-scan.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="8" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="B238" s="8" t="inlineStr">
+        <is>
+          <t>NVIDIA</t>
+        </is>
+      </c>
+      <c r="C238" s="8" t="inlineStr">
+        <is>
+          <t>sells GPUs to</t>
+        </is>
+      </c>
+      <c r="D238" s="8" t="inlineStr">
+        <is>
+          <t>SPCX</t>
+        </is>
+      </c>
+      <c r="E238" s="8" t="inlineStr">
+        <is>
+          <t>SpaceX (Colossus compute)</t>
+        </is>
+      </c>
+      <c r="F238" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G238" s="8" t="inlineStr">
+        <is>
+          <t>(FACT, X-scan 2026-06-05): SpaceX Colossus deploys ~110k NVIDIA GPUs to serve the Google compute contract (?) Colossus usually attributed to xAI</t>
+        </is>
+      </c>
+      <c r="H238" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="I238" s="8" t="inlineStr">
+        <is>
+          <t>X-Reports/2026-06-05-2004-x-scan.md</t>
         </is>
       </c>
     </row>
@@ -15099,7 +15797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15151,36 +15849,36 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F2" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T_NET</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Optical &amp; Networking Buildout</t>
+          <t>TSMC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Demand Driver / Theme</t>
+          <t>Foundry / Manufacturing</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E3" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
         <v>19</v>
@@ -15189,27 +15887,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>T_NET</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TSMC</t>
+          <t>Optical &amp; Networking Buildout</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Foundry / Manufacturing</t>
+          <t>Demand Driver / Theme</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="F4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -15232,10 +15930,10 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -15437,114 +16135,114 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
         <v>8</v>
       </c>
       <c r="F13" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Marvell</t>
+          <t>Intel</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Chip Designers (Accelerators/Networking)</t>
+          <t>Foundry / Manufacturing</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Intel</t>
+          <t>Arm Holdings</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Foundry / Manufacturing</t>
+          <t>EDA &amp; IP</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>T_HBM</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HBM Demand</t>
+          <t>Marvell</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Demand Driver / Theme</t>
+          <t>Chip Designers (Accelerators/Networking)</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>T_CHINA</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>China Indigenous AI Buildout</t>
+          <t>Micron</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Demand Driver / Theme</t>
+          <t>Memory (HBM/DRAM)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
         <v>7</v>
@@ -15553,76 +16251,76 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>T_HBM</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>HBM Demand</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment</t>
+          <t>Demand Driver / Theme</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>T_CHINA</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Micron</t>
+          <t>China Indigenous AI Buildout</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Memory (HBM/DRAM)</t>
+          <t>Demand Driver / Theme</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Vertiv</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Power &amp; Cooling Equipment</t>
+          <t>Semiconductor Equipment</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>6</v>
@@ -15631,17 +16329,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>T_GLASS</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Glass Core Substrate</t>
+          <t>Meta Platforms</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Demand Driver / Theme</t>
+          <t>Hyperscalers / Cloud</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -15657,128 +16355,128 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Coherent</t>
+          <t>Oracle</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>Hyperscalers / Cloud</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>OPENAI</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Fabrinet</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>AI Labs / Model Developers</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Arista Networks</t>
+          <t>Vertiv</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Networking Systems</t>
+          <t>Power &amp; Cooling Equipment</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>T_GLASS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Supermicro</t>
+          <t>Glass Core Substrate</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Servers &amp; ODM/OEM</t>
+          <t>Demand Driver / Theme</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Meta Platforms</t>
+          <t>Coherent</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hyperscalers / Cloud</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E26" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
         <v>5</v>
@@ -15787,24 +16485,24 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Oracle</t>
+          <t>Fabrinet</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Hyperscalers / Cloud</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="n">
         <v>0</v>
-      </c>
-      <c r="E27" t="n">
-        <v>5</v>
       </c>
       <c r="F27" t="n">
         <v>5</v>
@@ -15813,24 +16511,24 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OPENAI</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Arista Networks</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AI Labs / Model Developers</t>
+          <t>Networking Systems</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" t="n">
         <v>5</v>
@@ -15839,24 +16537,24 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Equinix</t>
+          <t>Supermicro</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Datacenter Infrastructure (REITs)</t>
+          <t>Servers &amp; ODM/OEM</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>5</v>
@@ -15865,24 +16563,24 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ANTHROPIC</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Credo Technology</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>AI Labs / Model Developers</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
         <v>5</v>
@@ -15891,24 +16589,24 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ILUVATAR</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Iluvatar CoreX</t>
+          <t>Equinix</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Chip Designers (Accelerators/Networking)</t>
+          <t>Datacenter Infrastructure (REITs)</t>
         </is>
       </c>
       <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
         <v>3</v>
-      </c>
-      <c r="E31" t="n">
-        <v>2</v>
       </c>
       <c r="F31" t="n">
         <v>5</v>
@@ -15917,24 +16615,24 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CoreWeave</t>
+          <t>Credo Technology</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Hyperscalers / Cloud</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
         <v>5</v>
@@ -15943,64 +16641,64 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>ILUVATAR</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Synopsys</t>
+          <t>Iluvatar CoreX</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>EDA &amp; IP</t>
+          <t>Chip Designers (Accelerators/Networking)</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Cadence</t>
+          <t>CoreWeave</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>EDA &amp; IP</t>
+          <t>Hyperscalers / Cloud</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E34" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Arm Holdings</t>
+          <t>Synopsys</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -16021,17 +16719,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Lumentum</t>
+          <t>Cadence</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>EDA &amp; IP</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -16047,24 +16745,24 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>SAMSUNG</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Cisco</t>
+          <t>Samsung Electronics</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Networking Systems</t>
+          <t>Foundry / Manufacturing</t>
         </is>
       </c>
       <c r="D37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" t="n">
         <v>1</v>
-      </c>
-      <c r="E37" t="n">
-        <v>3</v>
       </c>
       <c r="F37" t="n">
         <v>4</v>
@@ -16073,24 +16771,24 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ANTHROPIC</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Lumentum</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AI Labs / Model Developers</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
         <v>4</v>
@@ -16099,24 +16797,24 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Digital Realty</t>
+          <t>Cisco</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Datacenter Infrastructure (REITs)</t>
+          <t>Networking Systems</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
         <v>4</v>
@@ -16125,17 +16823,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Digital Realty</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Hyperscalers / Cloud</t>
+          <t>Datacenter Infrastructure (REITs)</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -16151,24 +16849,24 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AAOI</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Applied Optoelectronics</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>Hyperscalers / Cloud</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>4</v>
@@ -16177,50 +16875,50 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>AAOI</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Lam Research</t>
+          <t>Applied Optoelectronics</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SAMSUNG</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Samsung Electronics</t>
+          <t>Lam Research</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Foundry / Manufacturing</t>
+          <t>Semiconductor Equipment</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
         <v>3</v>
@@ -16307,17 +17005,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>FOXCONN</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Eaton</t>
+          <t>Foxconn (Hon Hai)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Power &amp; Cooling Equipment</t>
+          <t>Servers &amp; ODM/OEM</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -16333,24 +17031,24 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Constellation Energy</t>
+          <t>Eaton</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Power Generation / Utilities</t>
+          <t>Power &amp; Cooling Equipment</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
         <v>3</v>
@@ -16359,12 +17057,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Vistra</t>
+          <t>Constellation Energy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -16385,12 +17083,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GE Vernova</t>
+          <t>Vistra</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -16399,10 +17097,10 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
         <v>3</v>
@@ -16411,24 +17109,24 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>T_COWOS</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CoWoS Advanced Packaging</t>
+          <t>GE Vernova</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Demand Driver / Theme</t>
+          <t>Power Generation / Utilities</t>
         </is>
       </c>
       <c r="D51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" t="n">
         <v>0</v>
-      </c>
-      <c r="E51" t="n">
-        <v>3</v>
       </c>
       <c r="F51" t="n">
         <v>3</v>
@@ -16437,24 +17135,24 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BOE</t>
+          <t>T_COWOS</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>BOE Technology</t>
+          <t>CoWoS Advanced Packaging</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Advanced Packaging / OSAT</t>
+          <t>Demand Driver / Theme</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F52" t="n">
         <v>3</v>
@@ -16463,12 +17161,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>BOE</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Corning</t>
+          <t>BOE Technology</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -16477,10 +17175,10 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F53" t="n">
         <v>3</v>
@@ -16489,12 +17187,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>INNOLUX</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Innolux</t>
+          <t>Corning</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -16503,10 +17201,10 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F54" t="n">
         <v>3</v>
@@ -16515,17 +17213,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>INNOLUX</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>Innolux</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Hyperscalers / Cloud</t>
+          <t>Advanced Packaging / OSAT</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -16541,24 +17239,24 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Bloom Energy</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Power &amp; Cooling Equipment</t>
+          <t>Hyperscalers / Cloud</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
         <v>3</v>
@@ -16567,17 +17265,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CLS</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Celestica</t>
+          <t>Bloom Energy</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Servers &amp; ODM/OEM</t>
+          <t>Power &amp; Cooling Equipment</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -16593,17 +17291,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>STM</t>
+          <t>CLS</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>STMicroelectronics</t>
+          <t>Celestica</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>Servers &amp; ODM/OEM</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -16619,12 +17317,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>STM</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Astera Labs</t>
+          <t>STMicroelectronics</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -16645,69 +17343,69 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Applied Materials</t>
+          <t>Astera Labs</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E60" t="n">
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>FOXCONN</t>
+          <t>SPCX</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Foxconn (Hon Hai)</t>
+          <t>SpaceX (Colossus compute)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Servers &amp; ODM/OEM</t>
+          <t>Hyperscalers / Cloud</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F61" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>FURUKAWA</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Furukawa Electric</t>
+          <t>Applied Materials</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>Semiconductor Equipment</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -16723,17 +17421,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>NAURA</t>
+          <t>FURUKAWA</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Naura Technology</t>
+          <t>Furukawa Electric</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -16749,12 +17447,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>AMEC</t>
+          <t>NAURA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Advanced Micro-Fabrication (AMEC)</t>
+          <t>Naura Technology</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -16775,17 +17473,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>METAX</t>
+          <t>AMEC</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MetaX</t>
+          <t>Advanced Micro-Fabrication (AMEC)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Chip Designers (Accelerators/Networking)</t>
+          <t>Semiconductor Equipment</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -16801,17 +17499,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CXMT</t>
+          <t>METAX</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ChangXin Memory (CXMT)</t>
+          <t>MetaX</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Memory (HBM/DRAM)</t>
+          <t>Chip Designers (Accelerators/Networking)</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -16827,17 +17525,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LUXSHARE</t>
+          <t>CXMT</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Luxshare Precision</t>
+          <t>ChangXin Memory (CXMT)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>Memory (HBM/DRAM)</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -16853,17 +17551,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>LUXSHARE</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Blackstone</t>
+          <t>Luxshare Precision</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Datacenter Infrastructure (REITs)</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -16879,17 +17577,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>AUO</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>AUO Corporation</t>
+          <t>Blackstone</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Advanced Packaging / OSAT</t>
+          <t>Datacenter Infrastructure (REITs)</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -16905,17 +17603,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CORZ</t>
+          <t>AUO</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Core Scientific</t>
+          <t>AUO Corporation</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Datacenter Infrastructure (REITs)</t>
+          <t>Advanced Packaging / OSAT</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -16931,12 +17629,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>APLD</t>
+          <t>CORZ</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Applied Digital</t>
+          <t>Core Scientific</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -16957,17 +17655,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>APLD</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>IBM</t>
+          <t>Applied Digital</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Chip Designers (Accelerators/Networking)</t>
+          <t>Datacenter Infrastructure (REITs)</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -16983,17 +17681,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>XFAB</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>X-FAB</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Foundry / Manufacturing</t>
+          <t>Chip Designers (Accelerators/Networking)</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -17009,17 +17707,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>POET</t>
+          <t>XFAB</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>POET Technologies</t>
+          <t>X-FAB</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>Foundry / Manufacturing</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -17035,12 +17733,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SIVE</t>
+          <t>POET</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Sivers Semiconductor</t>
+          <t>POET Technologies</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -17061,24 +17759,24 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>SIVE</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>GlobalFoundries</t>
+          <t>Sivers Semiconductor</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Foundry / Manufacturing</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E76" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F76" t="n">
         <v>2</v>
@@ -17087,17 +17785,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Qualcomm</t>
+          <t>GlobalFoundries</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Chip Designers (Accelerators/Networking)</t>
+          <t>Foundry / Manufacturing</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -17113,12 +17811,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MTK</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MediaTek</t>
+          <t>Qualcomm</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -17127,10 +17825,10 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F78" t="n">
         <v>2</v>
@@ -17139,17 +17837,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>AYAR</t>
+          <t>MTK</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Ayar Labs</t>
+          <t>MediaTek</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>Chip Designers (Accelerators/Networking)</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -17165,17 +17863,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>NANYA</t>
+          <t>AYAR</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Nanya Technology</t>
+          <t>Ayar Labs</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Memory (HBM/DRAM)</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -17191,17 +17889,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SMTC</t>
+          <t>NANYA</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Semtech</t>
+          <t>Nanya Technology</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>Memory (HBM/DRAM)</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -17217,50 +17915,50 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>SMTC</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>KLA Corporation</t>
+          <t>Semtech</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E82" t="n">
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Hewlett Packard Enterprise</t>
+          <t>KLA Corporation</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Servers &amp; ODM/OEM</t>
+          <t>Semiconductor Equipment</t>
         </is>
       </c>
       <c r="D83" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" t="n">
         <v>0</v>
-      </c>
-      <c r="E83" t="n">
-        <v>1</v>
       </c>
       <c r="F83" t="n">
         <v>1</v>
@@ -17269,17 +17967,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>T_COOL</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Liquid Cooling Adoption</t>
+          <t>Hewlett Packard Enterprise</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Demand Driver / Theme</t>
+          <t>Servers &amp; ODM/OEM</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -17295,24 +17993,24 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ALPHAWAVE</t>
+          <t>T_COOL</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Alphawave Semi</t>
+          <t>Liquid Cooling Adoption</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Optical &amp; Interconnect</t>
+          <t>Demand Driver / Theme</t>
         </is>
       </c>
       <c r="D85" t="n">
+        <v>0</v>
+      </c>
+      <c r="E85" t="n">
         <v>1</v>
-      </c>
-      <c r="E85" t="n">
-        <v>0</v>
       </c>
       <c r="F85" t="n">
         <v>1</v>
@@ -17321,17 +18019,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>ALPHAWAVE</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Alphawave Semi</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Power &amp; Cooling Equipment</t>
+          <t>Optical &amp; Interconnect</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -17347,12 +18045,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Analog Devices</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -17373,17 +18071,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>YMTC</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Yangtze Memory (YMTC)</t>
+          <t>Analog Devices</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Memory (HBM/DRAM)</t>
+          <t>Power &amp; Cooling Equipment</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -17399,24 +18097,24 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>YMTC</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Huawei</t>
+          <t>Yangtze Memory (YMTC)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Chip Designers (Accelerators/Networking)</t>
+          <t>Memory (HBM/DRAM)</t>
         </is>
       </c>
       <c r="D89" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" t="n">
         <v>0</v>
-      </c>
-      <c r="E89" t="n">
-        <v>1</v>
       </c>
       <c r="F89" t="n">
         <v>1</v>
@@ -17425,24 +18123,24 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Teradyne</t>
+          <t>Huawei</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Semiconductor Equipment</t>
+          <t>Chip Designers (Accelerators/Networking)</t>
         </is>
       </c>
       <c r="D90" t="n">
+        <v>0</v>
+      </c>
+      <c r="E90" t="n">
         <v>1</v>
-      </c>
-      <c r="E90" t="n">
-        <v>0</v>
       </c>
       <c r="F90" t="n">
         <v>1</v>
@@ -17451,12 +18149,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>XLIGHT</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>XLight</t>
+          <t>Teradyne</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -17477,17 +18175,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>XLIGHT</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Sandisk</t>
+          <t>XLight</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Memory (HBM/DRAM)</t>
+          <t>Semiconductor Equipment</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -17503,17 +18201,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CIFR</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Cipher Mining</t>
+          <t>Sandisk</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Datacenter Infrastructure (REITs)</t>
+          <t>Memory (HBM/DRAM)</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -17529,24 +18227,24 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>XAI</t>
+          <t>CIFR</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>xAI</t>
+          <t>Cipher Mining</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>AI Labs / Model Developers</t>
+          <t>Datacenter Infrastructure (REITs)</t>
         </is>
       </c>
       <c r="D94" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" t="n">
         <v>0</v>
-      </c>
-      <c r="E94" t="n">
-        <v>1</v>
       </c>
       <c r="F94" t="n">
         <v>1</v>
@@ -17555,26 +18253,104 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
+          <t>XAI</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>AI Labs / Model Developers</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E95" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
           <t>ENTG</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>Entegris</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>Semiconductor Equipment</t>
         </is>
       </c>
-      <c r="D95" t="n">
+      <c r="D96" t="n">
         <v>1</v>
       </c>
-      <c r="E95" t="n">
+      <c r="E96" t="n">
         <v>0</v>
       </c>
-      <c r="F95" t="n">
+      <c r="F96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>SAMBANOVA</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>SambaNova Systems</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Chip Designers (Accelerators/Networking)</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" t="n">
+        <v>0</v>
+      </c>
+      <c r="F97" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>BYTEDANCE</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>ByteDance</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Hyperscalers / Cloud</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>0</v>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>